<commit_message>
Add unit test for outlier detection in Batch processing
- Implemented a new test `test_outlier_detection` to verify the identification of outliers in the Batch class.
- The test checks for three types of outliers: variance, amplitude, and range.
- Variance and amplitude outliers are flagged immediately, while range outliers are checked post-processing.
- Utilized mock data to simulate different outlier scenarios and validate alert generation.
</commit_message>
<xml_diff>
--- a/Water_2H_Report.xlsx
+++ b/Water_2H_Report.xlsx
@@ -495,13 +495,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-73.63</v>
+        <v>-74.56</v>
       </c>
       <c r="C5" t="n">
-        <v>1.72</v>
+        <v>1.55</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">

</xml_diff>